<commit_message>
Implement Rainbow bomb gauge system (original PokoPang mechanic)
- Add BombType.Rainbow and gauge-based spawning
- Remove PokoBlockSubtype.Rainbow (Rainbow is now a bomb, not a tile)
- Rainbow gauge fills proportionally to blocks cleared per chain
- Full gauge spawns a Rainbow bomb tile on the board
- Rainbow bomb detonation clears all tiles of the most common color
- Add rainbow gauge bar to screen HUD
- Remove old IsRainbow/ActivateRainbowTile code paths
</commit_message>
<xml_diff>
--- a/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
+++ b/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
@@ -474,10 +474,8 @@
           <t>Snow Imp</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="C2" t="n">
+        <v>45</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -506,10 +504,8 @@
           <t>Pebble Guard</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="C3" t="n">
+        <v>60</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -539,7 +535,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -568,10 +564,8 @@
           <t>Frost Larva</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
+      <c r="C5" t="n">
+        <v>75</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -601,7 +595,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -629,7 +623,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D7" t="n">
         <v>55</v>
@@ -655,7 +649,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="D8" t="n">
         <v>85</v>
@@ -681,7 +675,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D9" t="n">
         <v>45</v>
@@ -707,7 +701,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D10" t="n">
         <v>70</v>
@@ -733,7 +727,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D11" t="n">
         <v>110</v>
@@ -808,10 +802,8 @@
           <t>Frost Queen</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
+      <c r="C2" t="n">
+        <v>240</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -836,7 +828,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="D3" t="n">
         <v>550</v>
@@ -859,7 +851,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>380</v>
       </c>
       <c r="D4" t="n">
         <v>600</v>
@@ -881,10 +873,8 @@
           <t>Frost Wyrm</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+      <c r="C5" t="n">
+        <v>480</v>
       </c>
       <c r="D5" t="n">
         <v>750</v>
@@ -906,10 +896,8 @@
           <t>Chaos Lord</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="C6" t="n">
+        <v>650</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adjust UI to PokoPang style: timer, boss HP, board layout
- Redesign top panel: large TIME display with red warning at <=10s
- Boss HP bar: red fill with boss name/HP text, wave label above
- Regular enemy HP bar: blue fill
- Remove AI designer HUD text from gameplay
- End panel: GAME CLEAR instead of TARGET CLEAR
- Board camera: more vertical room (+3.5f offset)
- Default tile types: 5→6 (adds Orange)
</commit_message>
<xml_diff>
--- a/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
+++ b/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
@@ -423,12 +423,12 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col width="7.48125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="13.78125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="2.8875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="9.84375" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6.43125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="6.95625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="16" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10" bestFit="1" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -757,11 +757,11 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col width="5.11875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="11.94375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="3.54375" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.7625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6.95625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10" bestFit="1" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -924,13 +924,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col width="5.11875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="5.64375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="8.6625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.36875" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="11.2875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="6.69375" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="6.95625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="10" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1144,11 +1144,11 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>

</xml_diff>

<commit_message>
Add enemy backgrounds, fix collapse/refill bugs, update portfolio evidence
- Add BoardBackgroundRenderer and enemy/boss background assets
- Fix drop animation sync execution causing misplaced tile warnings
- Fix fixed obstacle position check in CompactColumns
- Update playtest analysis with full telemetry (29 moves, 43895 score)
- Update portfolio milestone with validation complete status
- Archive enemy-rotation-backgrounds OpenSpec change
</commit_message>
<xml_diff>
--- a/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
+++ b/Assets/PokoPuzzle/Data/Excel/GameData.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Enemy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Boss" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Skill" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="BalanceProfile" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boss" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BalanceProfile" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,11 @@
           <t>PortraitPath</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>BackgroundPath</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -504,6 +509,11 @@
           <t>EnemyPortraits/frostbinder_imp</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/frostbinder_imp</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -541,6 +551,11 @@
           <t>EnemyPortraits/rime_wisp</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/rime_wisp</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -578,6 +593,11 @@
           <t>EnemyPortraits/granite_mite</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/granite_mite</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -615,6 +635,11 @@
           <t>EnemyPortraits/crystal_guard</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/crystal_guard</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -652,6 +677,11 @@
           <t>EnemyPortraits/prism_bat</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/prism_bat</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -689,6 +719,11 @@
           <t>EnemyPortraits/chroma_shifter</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/chroma_shifter</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -726,6 +761,11 @@
           <t>EnemyPortraits/icebound_larva</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/icebound_larva</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -763,6 +803,11 @@
           <t>EnemyPortraits/stonehide_serpent</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/stonehide_serpent</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -800,6 +845,11 @@
           <t>EnemyPortraits/hue_imp</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/hue_imp</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -835,6 +885,11 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>EnemyPortraits/chroma_wisp</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/chroma_wisp</t>
         </is>
       </c>
     </row>
@@ -868,6 +923,11 @@
           <t>EnemyPortraits/basalt_crawler</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/basalt_crawler</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -897,6 +957,11 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>EnemyPortraits/onyx_gargoyle</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/onyx_gargoyle</t>
         </is>
       </c>
     </row>
@@ -911,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col width="8" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -952,6 +1017,11 @@
           <t>PortraitPath</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>BackgroundPath</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -984,6 +1054,11 @@
           <t>EnemyPortraits/frostbind_queen</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/frostbind_queen</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1016,6 +1091,11 @@
           <t>EnemyPortraits/stoneheart_golem</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/stoneheart_golem</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1048,6 +1128,11 @@
           <t>EnemyPortraits/prism_trickster</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/prism_trickster</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1080,6 +1165,11 @@
           <t>EnemyPortraits/blizzard_wyrm</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/blizzard_wyrm</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1110,6 +1200,11 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>EnemyPortraits/chroma_overlord</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/chroma_overlord</t>
         </is>
       </c>
     </row>
@@ -1136,6 +1231,11 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>EnemyPortraits/obsidian_basilisk</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>EnemyBackgrounds/obsidian_basilisk</t>
         </is>
       </c>
     </row>

</xml_diff>